<commit_message>
Checkliste und Zeitplan bearbeitet
</commit_message>
<xml_diff>
--- a/Dokumentation/Checkliste.xlsx
+++ b/Dokumentation/Checkliste.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sluz-my.sharepoint.com/personal/kuno_schuerch_sluz_ch/Documents/431/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\03BBZW\02Semester\M431\Projekt\BBZW-M431-Wiki\Dokumentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{40E32FD5-74D1-4DF5-B07C-D0FDAACB5ED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1D6A4AE-9940-4FF9-8CCF-68331A2144D6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07003136-728C-44B7-8565-AC4F19EB58C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33300" yWindow="2700" windowWidth="25035" windowHeight="17100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Checkliste" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="-Disclaimer-" sheetId="2" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Checkliste!$B$2:$G$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Checkliste!$B$2:$G$10</definedName>
   </definedNames>
   <calcPr calcId="140000"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
   <si>
     <t>Status</t>
   </si>
@@ -62,18 +62,6 @@
     <t>Fertig</t>
   </si>
   <si>
-    <t>Aufgabe 1</t>
-  </si>
-  <si>
-    <t>Aufgabe 2</t>
-  </si>
-  <si>
-    <t>Aufgabe 3</t>
-  </si>
-  <si>
-    <t>Aufgabe 4</t>
-  </si>
-  <si>
     <t>Gestartet</t>
   </si>
   <si>
@@ -86,7 +74,28 @@
     <t>Tief</t>
   </si>
   <si>
-    <t>Lernende/r 1</t>
+    <t>Projekt abgeben</t>
+  </si>
+  <si>
+    <t>Alle</t>
+  </si>
+  <si>
+    <t>Ist ein Sonntag</t>
+  </si>
+  <si>
+    <t>To Do</t>
+  </si>
+  <si>
+    <t>Webseite aufsetzetn</t>
+  </si>
+  <si>
+    <t>Inhalt für Webseite schreiben</t>
+  </si>
+  <si>
+    <t>MC Demo Server aufsetzetn</t>
+  </si>
+  <si>
+    <t>MC Demo Server testen</t>
   </si>
 </sst>
 </file>
@@ -231,12 +240,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -266,9 +272,6 @@
     <xf numFmtId="14" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -281,7 +284,27 @@
     <cellStyle name="Normal 2" xfId="2" xr:uid="{6D054895-97CA-45CE-99CE-3DACCCD181B9}"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -639,7 +662,7 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:BN376"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="3.5" customWidth="1"/>
     <col min="2" max="2" width="52" customWidth="1"/>
@@ -650,15 +673,15 @@
     <col min="8" max="8" width="4.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:66" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="8" t="s">
+    <row r="1" spans="1:66" ht="50.1" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="9"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
@@ -719,24 +742,24 @@
       <c r="BM1" s="1"/>
       <c r="BN1" s="1"/>
     </row>
-    <row r="2" spans="1:66" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:66" ht="33" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="1"/>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="13" t="s">
         <v>8</v>
       </c>
       <c r="H2" s="1"/>
@@ -799,22 +822,16 @@
       <c r="BM2" s="1"/>
       <c r="BN2" s="1"/>
     </row>
-    <row r="3" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A3" s="1"/>
-      <c r="B3" s="11" t="s">
-        <v>10</v>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="11">
+        <v>46160</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="12">
-        <v>45994</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" s="11"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
@@ -875,18 +892,16 @@
       <c r="BM3" s="1"/>
       <c r="BN3" s="1"/>
     </row>
-    <row r="4" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A4" s="1"/>
-      <c r="B4" s="11" t="s">
-        <v>11</v>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="11">
+        <v>46167</v>
       </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="12"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
@@ -947,18 +962,16 @@
       <c r="BM4" s="1"/>
       <c r="BN4" s="1"/>
     </row>
-    <row r="5" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A5" s="1"/>
-      <c r="B5" s="11" t="s">
-        <v>12</v>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="11">
+        <v>46174</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" s="12"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
@@ -1019,16 +1032,16 @@
       <c r="BM5" s="1"/>
       <c r="BN5" s="1"/>
     </row>
-    <row r="6" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A6" s="1"/>
-      <c r="B6" s="11" t="s">
-        <v>13</v>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="11">
+        <v>46181</v>
       </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
@@ -1089,14 +1102,26 @@
       <c r="BM6" s="1"/>
       <c r="BN6" s="1"/>
     </row>
-    <row r="7" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A7" s="1"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
+      <c r="B7" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="11">
+        <v>46187</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>16</v>
+      </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
@@ -1157,14 +1182,16 @@
       <c r="BM7" s="1"/>
       <c r="BN7" s="1"/>
     </row>
-    <row r="8" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A8" s="1"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
+      <c r="B8" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
@@ -1225,14 +1252,16 @@
       <c r="BM8" s="1"/>
       <c r="BN8" s="1"/>
     </row>
-    <row r="9" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A9" s="1"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
+      <c r="B9" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
@@ -1293,14 +1322,15 @@
       <c r="BM9" s="1"/>
       <c r="BN9" s="1"/>
     </row>
-    <row r="10" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A10" s="1"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
+      <c r="B10" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
@@ -1361,14 +1391,16 @@
       <c r="BM10" s="1"/>
       <c r="BN10" s="1"/>
     </row>
-    <row r="11" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A11" s="1"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
+      <c r="B11" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
@@ -1429,14 +1461,14 @@
       <c r="BM11" s="1"/>
       <c r="BN11" s="1"/>
     </row>
-    <row r="12" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A12" s="1"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
@@ -1497,14 +1529,14 @@
       <c r="BM12" s="1"/>
       <c r="BN12" s="1"/>
     </row>
-    <row r="13" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A13" s="1"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
@@ -1565,14 +1597,14 @@
       <c r="BM13" s="1"/>
       <c r="BN13" s="1"/>
     </row>
-    <row r="14" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A14" s="1"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
@@ -1633,14 +1665,14 @@
       <c r="BM14" s="1"/>
       <c r="BN14" s="1"/>
     </row>
-    <row r="15" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A15" s="1"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
@@ -1701,14 +1733,14 @@
       <c r="BM15" s="1"/>
       <c r="BN15" s="1"/>
     </row>
-    <row r="16" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A16" s="1"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
@@ -1769,14 +1801,14 @@
       <c r="BM16" s="1"/>
       <c r="BN16" s="1"/>
     </row>
-    <row r="17" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A17" s="1"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
@@ -1837,14 +1869,14 @@
       <c r="BM17" s="1"/>
       <c r="BN17" s="1"/>
     </row>
-    <row r="18" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A18" s="1"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
@@ -1905,14 +1937,13 @@
       <c r="BM18" s="1"/>
       <c r="BN18" s="1"/>
     </row>
-    <row r="19" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A19" s="1"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
@@ -1973,14 +2004,14 @@
       <c r="BM19" s="1"/>
       <c r="BN19" s="1"/>
     </row>
-    <row r="20" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A20" s="1"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
@@ -2041,14 +2072,14 @@
       <c r="BM20" s="1"/>
       <c r="BN20" s="1"/>
     </row>
-    <row r="21" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A21" s="1"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
@@ -2109,14 +2140,14 @@
       <c r="BM21" s="1"/>
       <c r="BN21" s="1"/>
     </row>
-    <row r="22" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A22" s="1"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
@@ -2177,14 +2208,14 @@
       <c r="BM22" s="1"/>
       <c r="BN22" s="1"/>
     </row>
-    <row r="23" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A23" s="1"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
@@ -2245,14 +2276,14 @@
       <c r="BM23" s="1"/>
       <c r="BN23" s="1"/>
     </row>
-    <row r="24" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A24" s="1"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
@@ -2313,14 +2344,14 @@
       <c r="BM24" s="1"/>
       <c r="BN24" s="1"/>
     </row>
-    <row r="25" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A25" s="1"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
       <c r="J25" s="1"/>
@@ -2381,14 +2412,14 @@
       <c r="BM25" s="1"/>
       <c r="BN25" s="1"/>
     </row>
-    <row r="26" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:66" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A26" s="1"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
@@ -2449,7 +2480,7 @@
       <c r="BM26" s="1"/>
       <c r="BN26" s="1"/>
     </row>
-    <row r="27" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
@@ -2511,7 +2542,7 @@
       <c r="BM27" s="1"/>
       <c r="BN27" s="1"/>
     </row>
-    <row r="28" spans="1:66" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:66" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -2579,7 +2610,7 @@
       <c r="BM28" s="1"/>
       <c r="BN28" s="1"/>
     </row>
-    <row r="29" spans="1:66" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:66" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -2647,7 +2678,7 @@
       <c r="BM29" s="1"/>
       <c r="BN29" s="1"/>
     </row>
-    <row r="30" spans="1:66" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:66" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -2715,7 +2746,7 @@
       <c r="BM30" s="1"/>
       <c r="BN30" s="1"/>
     </row>
-    <row r="31" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -2783,7 +2814,7 @@
       <c r="BM31" s="1"/>
       <c r="BN31" s="1"/>
     </row>
-    <row r="32" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -2851,7 +2882,7 @@
       <c r="BM32" s="1"/>
       <c r="BN32" s="1"/>
     </row>
-    <row r="33" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -2919,7 +2950,7 @@
       <c r="BM33" s="1"/>
       <c r="BN33" s="1"/>
     </row>
-    <row r="34" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -2987,7 +3018,7 @@
       <c r="BM34" s="1"/>
       <c r="BN34" s="1"/>
     </row>
-    <row r="35" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -3055,7 +3086,7 @@
       <c r="BM35" s="1"/>
       <c r="BN35" s="1"/>
     </row>
-    <row r="36" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -3123,7 +3154,7 @@
       <c r="BM36" s="1"/>
       <c r="BN36" s="1"/>
     </row>
-    <row r="37" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -3191,7 +3222,7 @@
       <c r="BM37" s="1"/>
       <c r="BN37" s="1"/>
     </row>
-    <row r="38" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -3259,7 +3290,7 @@
       <c r="BM38" s="1"/>
       <c r="BN38" s="1"/>
     </row>
-    <row r="39" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -3327,7 +3358,7 @@
       <c r="BM39" s="1"/>
       <c r="BN39" s="1"/>
     </row>
-    <row r="40" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -3395,7 +3426,7 @@
       <c r="BM40" s="1"/>
       <c r="BN40" s="1"/>
     </row>
-    <row r="41" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -3463,7 +3494,7 @@
       <c r="BM41" s="1"/>
       <c r="BN41" s="1"/>
     </row>
-    <row r="42" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -3531,7 +3562,7 @@
       <c r="BM42" s="1"/>
       <c r="BN42" s="1"/>
     </row>
-    <row r="43" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -3599,7 +3630,7 @@
       <c r="BM43" s="1"/>
       <c r="BN43" s="1"/>
     </row>
-    <row r="44" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -3667,7 +3698,7 @@
       <c r="BM44" s="1"/>
       <c r="BN44" s="1"/>
     </row>
-    <row r="45" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -3735,7 +3766,7 @@
       <c r="BM45" s="1"/>
       <c r="BN45" s="1"/>
     </row>
-    <row r="46" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -3803,7 +3834,7 @@
       <c r="BM46" s="1"/>
       <c r="BN46" s="1"/>
     </row>
-    <row r="47" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -3871,7 +3902,7 @@
       <c r="BM47" s="1"/>
       <c r="BN47" s="1"/>
     </row>
-    <row r="48" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -3939,7 +3970,7 @@
       <c r="BM48" s="1"/>
       <c r="BN48" s="1"/>
     </row>
-    <row r="49" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -4007,7 +4038,7 @@
       <c r="BM49" s="1"/>
       <c r="BN49" s="1"/>
     </row>
-    <row r="50" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -4075,7 +4106,7 @@
       <c r="BM50" s="1"/>
       <c r="BN50" s="1"/>
     </row>
-    <row r="51" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
@@ -4143,7 +4174,7 @@
       <c r="BM51" s="1"/>
       <c r="BN51" s="1"/>
     </row>
-    <row r="52" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
@@ -4211,7 +4242,7 @@
       <c r="BM52" s="1"/>
       <c r="BN52" s="1"/>
     </row>
-    <row r="53" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
@@ -4279,7 +4310,7 @@
       <c r="BM53" s="1"/>
       <c r="BN53" s="1"/>
     </row>
-    <row r="54" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
@@ -4347,7 +4378,7 @@
       <c r="BM54" s="1"/>
       <c r="BN54" s="1"/>
     </row>
-    <row r="55" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -4415,7 +4446,7 @@
       <c r="BM55" s="1"/>
       <c r="BN55" s="1"/>
     </row>
-    <row r="56" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
@@ -4483,7 +4514,7 @@
       <c r="BM56" s="1"/>
       <c r="BN56" s="1"/>
     </row>
-    <row r="57" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
@@ -4551,7 +4582,7 @@
       <c r="BM57" s="1"/>
       <c r="BN57" s="1"/>
     </row>
-    <row r="58" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
@@ -4619,7 +4650,7 @@
       <c r="BM58" s="1"/>
       <c r="BN58" s="1"/>
     </row>
-    <row r="59" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
@@ -4687,7 +4718,7 @@
       <c r="BM59" s="1"/>
       <c r="BN59" s="1"/>
     </row>
-    <row r="60" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
@@ -4755,7 +4786,7 @@
       <c r="BM60" s="1"/>
       <c r="BN60" s="1"/>
     </row>
-    <row r="61" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A61" s="1"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
@@ -4823,7 +4854,7 @@
       <c r="BM61" s="1"/>
       <c r="BN61" s="1"/>
     </row>
-    <row r="62" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
@@ -4891,7 +4922,7 @@
       <c r="BM62" s="1"/>
       <c r="BN62" s="1"/>
     </row>
-    <row r="63" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
@@ -4959,7 +4990,7 @@
       <c r="BM63" s="1"/>
       <c r="BN63" s="1"/>
     </row>
-    <row r="64" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
@@ -5027,7 +5058,7 @@
       <c r="BM64" s="1"/>
       <c r="BN64" s="1"/>
     </row>
-    <row r="65" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A65" s="1"/>
       <c r="B65" s="1"/>
       <c r="C65" s="1"/>
@@ -5095,7 +5126,7 @@
       <c r="BM65" s="1"/>
       <c r="BN65" s="1"/>
     </row>
-    <row r="66" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A66" s="1"/>
       <c r="B66" s="1"/>
       <c r="C66" s="1"/>
@@ -5163,7 +5194,7 @@
       <c r="BM66" s="1"/>
       <c r="BN66" s="1"/>
     </row>
-    <row r="67" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A67" s="1"/>
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
@@ -5231,7 +5262,7 @@
       <c r="BM67" s="1"/>
       <c r="BN67" s="1"/>
     </row>
-    <row r="68" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A68" s="1"/>
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
@@ -5299,7 +5330,7 @@
       <c r="BM68" s="1"/>
       <c r="BN68" s="1"/>
     </row>
-    <row r="69" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A69" s="1"/>
       <c r="B69" s="1"/>
       <c r="C69" s="1"/>
@@ -5367,7 +5398,7 @@
       <c r="BM69" s="1"/>
       <c r="BN69" s="1"/>
     </row>
-    <row r="70" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A70" s="1"/>
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
@@ -5435,7 +5466,7 @@
       <c r="BM70" s="1"/>
       <c r="BN70" s="1"/>
     </row>
-    <row r="71" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A71" s="1"/>
       <c r="B71" s="1"/>
       <c r="C71" s="1"/>
@@ -5503,7 +5534,7 @@
       <c r="BM71" s="1"/>
       <c r="BN71" s="1"/>
     </row>
-    <row r="72" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A72" s="1"/>
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
@@ -5571,7 +5602,7 @@
       <c r="BM72" s="1"/>
       <c r="BN72" s="1"/>
     </row>
-    <row r="73" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A73" s="1"/>
       <c r="B73" s="1"/>
       <c r="C73" s="1"/>
@@ -5639,7 +5670,7 @@
       <c r="BM73" s="1"/>
       <c r="BN73" s="1"/>
     </row>
-    <row r="74" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A74" s="1"/>
       <c r="B74" s="1"/>
       <c r="C74" s="1"/>
@@ -5707,7 +5738,7 @@
       <c r="BM74" s="1"/>
       <c r="BN74" s="1"/>
     </row>
-    <row r="75" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A75" s="1"/>
       <c r="B75" s="1"/>
       <c r="C75" s="1"/>
@@ -5775,7 +5806,7 @@
       <c r="BM75" s="1"/>
       <c r="BN75" s="1"/>
     </row>
-    <row r="76" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A76" s="1"/>
       <c r="B76" s="1"/>
       <c r="C76" s="1"/>
@@ -5843,7 +5874,7 @@
       <c r="BM76" s="1"/>
       <c r="BN76" s="1"/>
     </row>
-    <row r="77" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A77" s="1"/>
       <c r="B77" s="1"/>
       <c r="C77" s="1"/>
@@ -5911,7 +5942,7 @@
       <c r="BM77" s="1"/>
       <c r="BN77" s="1"/>
     </row>
-    <row r="78" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A78" s="1"/>
       <c r="B78" s="1"/>
       <c r="C78" s="1"/>
@@ -5979,7 +6010,7 @@
       <c r="BM78" s="1"/>
       <c r="BN78" s="1"/>
     </row>
-    <row r="79" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
@@ -6047,7 +6078,7 @@
       <c r="BM79" s="1"/>
       <c r="BN79" s="1"/>
     </row>
-    <row r="80" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A80" s="1"/>
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
@@ -6115,7 +6146,7 @@
       <c r="BM80" s="1"/>
       <c r="BN80" s="1"/>
     </row>
-    <row r="81" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A81" s="1"/>
       <c r="B81" s="1"/>
       <c r="C81" s="1"/>
@@ -6183,7 +6214,7 @@
       <c r="BM81" s="1"/>
       <c r="BN81" s="1"/>
     </row>
-    <row r="82" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A82" s="1"/>
       <c r="B82" s="1"/>
       <c r="C82" s="1"/>
@@ -6251,7 +6282,7 @@
       <c r="BM82" s="1"/>
       <c r="BN82" s="1"/>
     </row>
-    <row r="83" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A83" s="1"/>
       <c r="B83" s="1"/>
       <c r="C83" s="1"/>
@@ -6319,7 +6350,7 @@
       <c r="BM83" s="1"/>
       <c r="BN83" s="1"/>
     </row>
-    <row r="84" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A84" s="1"/>
       <c r="B84" s="1"/>
       <c r="C84" s="1"/>
@@ -6387,7 +6418,7 @@
       <c r="BM84" s="1"/>
       <c r="BN84" s="1"/>
     </row>
-    <row r="85" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A85" s="1"/>
       <c r="B85" s="1"/>
       <c r="C85" s="1"/>
@@ -6455,7 +6486,7 @@
       <c r="BM85" s="1"/>
       <c r="BN85" s="1"/>
     </row>
-    <row r="86" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A86" s="1"/>
       <c r="B86" s="1"/>
       <c r="C86" s="1"/>
@@ -6523,7 +6554,7 @@
       <c r="BM86" s="1"/>
       <c r="BN86" s="1"/>
     </row>
-    <row r="87" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A87" s="1"/>
       <c r="B87" s="1"/>
       <c r="C87" s="1"/>
@@ -6591,7 +6622,7 @@
       <c r="BM87" s="1"/>
       <c r="BN87" s="1"/>
     </row>
-    <row r="88" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A88" s="1"/>
       <c r="B88" s="1"/>
       <c r="C88" s="1"/>
@@ -6659,7 +6690,7 @@
       <c r="BM88" s="1"/>
       <c r="BN88" s="1"/>
     </row>
-    <row r="89" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A89" s="1"/>
       <c r="B89" s="1"/>
       <c r="C89" s="1"/>
@@ -6727,7 +6758,7 @@
       <c r="BM89" s="1"/>
       <c r="BN89" s="1"/>
     </row>
-    <row r="90" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A90" s="1"/>
       <c r="B90" s="1"/>
       <c r="C90" s="1"/>
@@ -6795,7 +6826,7 @@
       <c r="BM90" s="1"/>
       <c r="BN90" s="1"/>
     </row>
-    <row r="91" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A91" s="1"/>
       <c r="B91" s="1"/>
       <c r="C91" s="1"/>
@@ -6863,7 +6894,7 @@
       <c r="BM91" s="1"/>
       <c r="BN91" s="1"/>
     </row>
-    <row r="92" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A92" s="1"/>
       <c r="B92" s="1"/>
       <c r="C92" s="1"/>
@@ -6931,7 +6962,7 @@
       <c r="BM92" s="1"/>
       <c r="BN92" s="1"/>
     </row>
-    <row r="93" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A93" s="1"/>
       <c r="B93" s="1"/>
       <c r="C93" s="1"/>
@@ -6999,7 +7030,7 @@
       <c r="BM93" s="1"/>
       <c r="BN93" s="1"/>
     </row>
-    <row r="94" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A94" s="1"/>
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
@@ -7067,7 +7098,7 @@
       <c r="BM94" s="1"/>
       <c r="BN94" s="1"/>
     </row>
-    <row r="95" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A95" s="1"/>
       <c r="B95" s="1"/>
       <c r="C95" s="1"/>
@@ -7135,7 +7166,7 @@
       <c r="BM95" s="1"/>
       <c r="BN95" s="1"/>
     </row>
-    <row r="96" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A96" s="1"/>
       <c r="B96" s="1"/>
       <c r="C96" s="1"/>
@@ -7203,7 +7234,7 @@
       <c r="BM96" s="1"/>
       <c r="BN96" s="1"/>
     </row>
-    <row r="97" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A97" s="1"/>
       <c r="B97" s="1"/>
       <c r="C97" s="1"/>
@@ -7271,7 +7302,7 @@
       <c r="BM97" s="1"/>
       <c r="BN97" s="1"/>
     </row>
-    <row r="98" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A98" s="1"/>
       <c r="B98" s="1"/>
       <c r="C98" s="1"/>
@@ -7339,7 +7370,7 @@
       <c r="BM98" s="1"/>
       <c r="BN98" s="1"/>
     </row>
-    <row r="99" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A99" s="1"/>
       <c r="B99" s="1"/>
       <c r="C99" s="1"/>
@@ -7407,7 +7438,7 @@
       <c r="BM99" s="1"/>
       <c r="BN99" s="1"/>
     </row>
-    <row r="100" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A100" s="1"/>
       <c r="B100" s="1"/>
       <c r="C100" s="1"/>
@@ -7475,7 +7506,7 @@
       <c r="BM100" s="1"/>
       <c r="BN100" s="1"/>
     </row>
-    <row r="101" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A101" s="1"/>
       <c r="B101" s="1"/>
       <c r="C101" s="1"/>
@@ -7543,7 +7574,7 @@
       <c r="BM101" s="1"/>
       <c r="BN101" s="1"/>
     </row>
-    <row r="102" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A102" s="1"/>
       <c r="B102" s="1"/>
       <c r="C102" s="1"/>
@@ -7611,7 +7642,7 @@
       <c r="BM102" s="1"/>
       <c r="BN102" s="1"/>
     </row>
-    <row r="103" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A103" s="1"/>
       <c r="B103" s="1"/>
       <c r="C103" s="1"/>
@@ -7679,7 +7710,7 @@
       <c r="BM103" s="1"/>
       <c r="BN103" s="1"/>
     </row>
-    <row r="104" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A104" s="1"/>
       <c r="B104" s="1"/>
       <c r="C104" s="1"/>
@@ -7747,7 +7778,7 @@
       <c r="BM104" s="1"/>
       <c r="BN104" s="1"/>
     </row>
-    <row r="105" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A105" s="1"/>
       <c r="B105" s="1"/>
       <c r="C105" s="1"/>
@@ -7815,7 +7846,7 @@
       <c r="BM105" s="1"/>
       <c r="BN105" s="1"/>
     </row>
-    <row r="106" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A106" s="1"/>
       <c r="B106" s="1"/>
       <c r="C106" s="1"/>
@@ -7883,7 +7914,7 @@
       <c r="BM106" s="1"/>
       <c r="BN106" s="1"/>
     </row>
-    <row r="107" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A107" s="1"/>
       <c r="B107" s="1"/>
       <c r="C107" s="1"/>
@@ -7951,7 +7982,7 @@
       <c r="BM107" s="1"/>
       <c r="BN107" s="1"/>
     </row>
-    <row r="108" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A108" s="1"/>
       <c r="B108" s="1"/>
       <c r="C108" s="1"/>
@@ -8019,7 +8050,7 @@
       <c r="BM108" s="1"/>
       <c r="BN108" s="1"/>
     </row>
-    <row r="109" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A109" s="1"/>
       <c r="B109" s="1"/>
       <c r="C109" s="1"/>
@@ -8087,7 +8118,7 @@
       <c r="BM109" s="1"/>
       <c r="BN109" s="1"/>
     </row>
-    <row r="110" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A110" s="1"/>
       <c r="B110" s="1"/>
       <c r="C110" s="1"/>
@@ -8155,7 +8186,7 @@
       <c r="BM110" s="1"/>
       <c r="BN110" s="1"/>
     </row>
-    <row r="111" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A111" s="1"/>
       <c r="B111" s="1"/>
       <c r="C111" s="1"/>
@@ -8223,7 +8254,7 @@
       <c r="BM111" s="1"/>
       <c r="BN111" s="1"/>
     </row>
-    <row r="112" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A112" s="1"/>
       <c r="B112" s="1"/>
       <c r="C112" s="1"/>
@@ -8291,7 +8322,7 @@
       <c r="BM112" s="1"/>
       <c r="BN112" s="1"/>
     </row>
-    <row r="113" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A113" s="1"/>
       <c r="B113" s="1"/>
       <c r="C113" s="1"/>
@@ -8359,7 +8390,7 @@
       <c r="BM113" s="1"/>
       <c r="BN113" s="1"/>
     </row>
-    <row r="114" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A114" s="1"/>
       <c r="B114" s="1"/>
       <c r="C114" s="1"/>
@@ -8427,7 +8458,7 @@
       <c r="BM114" s="1"/>
       <c r="BN114" s="1"/>
     </row>
-    <row r="115" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A115" s="1"/>
       <c r="B115" s="1"/>
       <c r="C115" s="1"/>
@@ -8495,7 +8526,7 @@
       <c r="BM115" s="1"/>
       <c r="BN115" s="1"/>
     </row>
-    <row r="116" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A116" s="1"/>
       <c r="B116" s="1"/>
       <c r="C116" s="1"/>
@@ -8563,7 +8594,7 @@
       <c r="BM116" s="1"/>
       <c r="BN116" s="1"/>
     </row>
-    <row r="117" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A117" s="1"/>
       <c r="B117" s="1"/>
       <c r="C117" s="1"/>
@@ -8631,7 +8662,7 @@
       <c r="BM117" s="1"/>
       <c r="BN117" s="1"/>
     </row>
-    <row r="118" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A118" s="1"/>
       <c r="B118" s="1"/>
       <c r="C118" s="1"/>
@@ -8699,7 +8730,7 @@
       <c r="BM118" s="1"/>
       <c r="BN118" s="1"/>
     </row>
-    <row r="119" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A119" s="1"/>
       <c r="B119" s="1"/>
       <c r="C119" s="1"/>
@@ -8767,7 +8798,7 @@
       <c r="BM119" s="1"/>
       <c r="BN119" s="1"/>
     </row>
-    <row r="120" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A120" s="1"/>
       <c r="B120" s="1"/>
       <c r="C120" s="1"/>
@@ -8835,7 +8866,7 @@
       <c r="BM120" s="1"/>
       <c r="BN120" s="1"/>
     </row>
-    <row r="121" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A121" s="1"/>
       <c r="B121" s="1"/>
       <c r="C121" s="1"/>
@@ -8903,7 +8934,7 @@
       <c r="BM121" s="1"/>
       <c r="BN121" s="1"/>
     </row>
-    <row r="122" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A122" s="1"/>
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
@@ -8971,7 +9002,7 @@
       <c r="BM122" s="1"/>
       <c r="BN122" s="1"/>
     </row>
-    <row r="123" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A123" s="1"/>
       <c r="B123" s="1"/>
       <c r="C123" s="1"/>
@@ -9039,7 +9070,7 @@
       <c r="BM123" s="1"/>
       <c r="BN123" s="1"/>
     </row>
-    <row r="124" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A124" s="1"/>
       <c r="B124" s="1"/>
       <c r="C124" s="1"/>
@@ -9107,7 +9138,7 @@
       <c r="BM124" s="1"/>
       <c r="BN124" s="1"/>
     </row>
-    <row r="125" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A125" s="1"/>
       <c r="B125" s="1"/>
       <c r="C125" s="1"/>
@@ -9175,7 +9206,7 @@
       <c r="BM125" s="1"/>
       <c r="BN125" s="1"/>
     </row>
-    <row r="126" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A126" s="1"/>
       <c r="B126" s="1"/>
       <c r="C126" s="1"/>
@@ -9243,7 +9274,7 @@
       <c r="BM126" s="1"/>
       <c r="BN126" s="1"/>
     </row>
-    <row r="127" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A127" s="1"/>
       <c r="B127" s="1"/>
       <c r="C127" s="1"/>
@@ -9311,7 +9342,7 @@
       <c r="BM127" s="1"/>
       <c r="BN127" s="1"/>
     </row>
-    <row r="128" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A128" s="1"/>
       <c r="B128" s="1"/>
       <c r="C128" s="1"/>
@@ -9379,7 +9410,7 @@
       <c r="BM128" s="1"/>
       <c r="BN128" s="1"/>
     </row>
-    <row r="129" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A129" s="1"/>
       <c r="B129" s="1"/>
       <c r="C129" s="1"/>
@@ -9447,7 +9478,7 @@
       <c r="BM129" s="1"/>
       <c r="BN129" s="1"/>
     </row>
-    <row r="130" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A130" s="1"/>
       <c r="B130" s="1"/>
       <c r="C130" s="1"/>
@@ -9515,7 +9546,7 @@
       <c r="BM130" s="1"/>
       <c r="BN130" s="1"/>
     </row>
-    <row r="131" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A131" s="1"/>
       <c r="B131" s="1"/>
       <c r="C131" s="1"/>
@@ -9583,7 +9614,7 @@
       <c r="BM131" s="1"/>
       <c r="BN131" s="1"/>
     </row>
-    <row r="132" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A132" s="1"/>
       <c r="B132" s="1"/>
       <c r="C132" s="1"/>
@@ -9651,7 +9682,7 @@
       <c r="BM132" s="1"/>
       <c r="BN132" s="1"/>
     </row>
-    <row r="133" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A133" s="1"/>
       <c r="B133" s="1"/>
       <c r="C133" s="1"/>
@@ -9719,7 +9750,7 @@
       <c r="BM133" s="1"/>
       <c r="BN133" s="1"/>
     </row>
-    <row r="134" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A134" s="1"/>
       <c r="B134" s="1"/>
       <c r="C134" s="1"/>
@@ -9787,7 +9818,7 @@
       <c r="BM134" s="1"/>
       <c r="BN134" s="1"/>
     </row>
-    <row r="135" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A135" s="1"/>
       <c r="B135" s="1"/>
       <c r="C135" s="1"/>
@@ -9855,7 +9886,7 @@
       <c r="BM135" s="1"/>
       <c r="BN135" s="1"/>
     </row>
-    <row r="136" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A136" s="1"/>
       <c r="B136" s="1"/>
       <c r="C136" s="1"/>
@@ -9923,7 +9954,7 @@
       <c r="BM136" s="1"/>
       <c r="BN136" s="1"/>
     </row>
-    <row r="137" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A137" s="1"/>
       <c r="B137" s="1"/>
       <c r="C137" s="1"/>
@@ -9991,7 +10022,7 @@
       <c r="BM137" s="1"/>
       <c r="BN137" s="1"/>
     </row>
-    <row r="138" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A138" s="1"/>
       <c r="B138" s="1"/>
       <c r="C138" s="1"/>
@@ -10059,7 +10090,7 @@
       <c r="BM138" s="1"/>
       <c r="BN138" s="1"/>
     </row>
-    <row r="139" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A139" s="1"/>
       <c r="B139" s="1"/>
       <c r="C139" s="1"/>
@@ -10127,7 +10158,7 @@
       <c r="BM139" s="1"/>
       <c r="BN139" s="1"/>
     </row>
-    <row r="140" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A140" s="1"/>
       <c r="B140" s="1"/>
       <c r="C140" s="1"/>
@@ -10195,7 +10226,7 @@
       <c r="BM140" s="1"/>
       <c r="BN140" s="1"/>
     </row>
-    <row r="141" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A141" s="1"/>
       <c r="B141" s="1"/>
       <c r="C141" s="1"/>
@@ -10263,7 +10294,7 @@
       <c r="BM141" s="1"/>
       <c r="BN141" s="1"/>
     </row>
-    <row r="142" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A142" s="1"/>
       <c r="B142" s="1"/>
       <c r="C142" s="1"/>
@@ -10331,7 +10362,7 @@
       <c r="BM142" s="1"/>
       <c r="BN142" s="1"/>
     </row>
-    <row r="143" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A143" s="1"/>
       <c r="B143" s="1"/>
       <c r="C143" s="1"/>
@@ -10399,7 +10430,7 @@
       <c r="BM143" s="1"/>
       <c r="BN143" s="1"/>
     </row>
-    <row r="144" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A144" s="1"/>
       <c r="B144" s="1"/>
       <c r="C144" s="1"/>
@@ -10467,7 +10498,7 @@
       <c r="BM144" s="1"/>
       <c r="BN144" s="1"/>
     </row>
-    <row r="145" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A145" s="1"/>
       <c r="B145" s="1"/>
       <c r="C145" s="1"/>
@@ -10535,7 +10566,7 @@
       <c r="BM145" s="1"/>
       <c r="BN145" s="1"/>
     </row>
-    <row r="146" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A146" s="1"/>
       <c r="B146" s="1"/>
       <c r="C146" s="1"/>
@@ -10603,7 +10634,7 @@
       <c r="BM146" s="1"/>
       <c r="BN146" s="1"/>
     </row>
-    <row r="147" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A147" s="1"/>
       <c r="B147" s="1"/>
       <c r="C147" s="1"/>
@@ -10671,7 +10702,7 @@
       <c r="BM147" s="1"/>
       <c r="BN147" s="1"/>
     </row>
-    <row r="148" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A148" s="1"/>
       <c r="B148" s="1"/>
       <c r="C148" s="1"/>
@@ -10739,7 +10770,7 @@
       <c r="BM148" s="1"/>
       <c r="BN148" s="1"/>
     </row>
-    <row r="149" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A149" s="1"/>
       <c r="B149" s="1"/>
       <c r="C149" s="1"/>
@@ -10807,7 +10838,7 @@
       <c r="BM149" s="1"/>
       <c r="BN149" s="1"/>
     </row>
-    <row r="150" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A150" s="1"/>
       <c r="B150" s="1"/>
       <c r="C150" s="1"/>
@@ -10875,7 +10906,7 @@
       <c r="BM150" s="1"/>
       <c r="BN150" s="1"/>
     </row>
-    <row r="151" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A151" s="1"/>
       <c r="B151" s="1"/>
       <c r="C151" s="1"/>
@@ -10943,7 +10974,7 @@
       <c r="BM151" s="1"/>
       <c r="BN151" s="1"/>
     </row>
-    <row r="152" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A152" s="1"/>
       <c r="B152" s="1"/>
       <c r="C152" s="1"/>
@@ -11011,7 +11042,7 @@
       <c r="BM152" s="1"/>
       <c r="BN152" s="1"/>
     </row>
-    <row r="153" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A153" s="1"/>
       <c r="B153" s="1"/>
       <c r="C153" s="1"/>
@@ -11079,7 +11110,7 @@
       <c r="BM153" s="1"/>
       <c r="BN153" s="1"/>
     </row>
-    <row r="154" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A154" s="1"/>
       <c r="B154" s="1"/>
       <c r="C154" s="1"/>
@@ -11147,7 +11178,7 @@
       <c r="BM154" s="1"/>
       <c r="BN154" s="1"/>
     </row>
-    <row r="155" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A155" s="1"/>
       <c r="B155" s="1"/>
       <c r="C155" s="1"/>
@@ -11215,7 +11246,7 @@
       <c r="BM155" s="1"/>
       <c r="BN155" s="1"/>
     </row>
-    <row r="156" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A156" s="1"/>
       <c r="B156" s="1"/>
       <c r="C156" s="1"/>
@@ -11283,7 +11314,7 @@
       <c r="BM156" s="1"/>
       <c r="BN156" s="1"/>
     </row>
-    <row r="157" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A157" s="1"/>
       <c r="B157" s="1"/>
       <c r="C157" s="1"/>
@@ -11351,7 +11382,7 @@
       <c r="BM157" s="1"/>
       <c r="BN157" s="1"/>
     </row>
-    <row r="158" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A158" s="1"/>
       <c r="B158" s="1"/>
       <c r="C158" s="1"/>
@@ -11419,7 +11450,7 @@
       <c r="BM158" s="1"/>
       <c r="BN158" s="1"/>
     </row>
-    <row r="159" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A159" s="1"/>
       <c r="B159" s="1"/>
       <c r="C159" s="1"/>
@@ -11487,7 +11518,7 @@
       <c r="BM159" s="1"/>
       <c r="BN159" s="1"/>
     </row>
-    <row r="160" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A160" s="1"/>
       <c r="B160" s="1"/>
       <c r="C160" s="1"/>
@@ -11555,7 +11586,7 @@
       <c r="BM160" s="1"/>
       <c r="BN160" s="1"/>
     </row>
-    <row r="161" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A161" s="1"/>
       <c r="B161" s="1"/>
       <c r="C161" s="1"/>
@@ -11623,7 +11654,7 @@
       <c r="BM161" s="1"/>
       <c r="BN161" s="1"/>
     </row>
-    <row r="162" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A162" s="1"/>
       <c r="B162" s="1"/>
       <c r="C162" s="1"/>
@@ -11691,7 +11722,7 @@
       <c r="BM162" s="1"/>
       <c r="BN162" s="1"/>
     </row>
-    <row r="163" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A163" s="1"/>
       <c r="B163" s="1"/>
       <c r="C163" s="1"/>
@@ -11759,7 +11790,7 @@
       <c r="BM163" s="1"/>
       <c r="BN163" s="1"/>
     </row>
-    <row r="164" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A164" s="1"/>
       <c r="B164" s="1"/>
       <c r="C164" s="1"/>
@@ -11827,7 +11858,7 @@
       <c r="BM164" s="1"/>
       <c r="BN164" s="1"/>
     </row>
-    <row r="165" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A165" s="1"/>
       <c r="B165" s="1"/>
       <c r="C165" s="1"/>
@@ -11895,7 +11926,7 @@
       <c r="BM165" s="1"/>
       <c r="BN165" s="1"/>
     </row>
-    <row r="166" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A166" s="1"/>
       <c r="B166" s="1"/>
       <c r="C166" s="1"/>
@@ -11963,7 +11994,7 @@
       <c r="BM166" s="1"/>
       <c r="BN166" s="1"/>
     </row>
-    <row r="167" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A167" s="1"/>
       <c r="B167" s="1"/>
       <c r="C167" s="1"/>
@@ -12031,7 +12062,7 @@
       <c r="BM167" s="1"/>
       <c r="BN167" s="1"/>
     </row>
-    <row r="168" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A168" s="1"/>
       <c r="B168" s="1"/>
       <c r="C168" s="1"/>
@@ -12099,7 +12130,7 @@
       <c r="BM168" s="1"/>
       <c r="BN168" s="1"/>
     </row>
-    <row r="169" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A169" s="1"/>
       <c r="B169" s="1"/>
       <c r="C169" s="1"/>
@@ -12167,7 +12198,7 @@
       <c r="BM169" s="1"/>
       <c r="BN169" s="1"/>
     </row>
-    <row r="170" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A170" s="1"/>
       <c r="B170" s="1"/>
       <c r="C170" s="1"/>
@@ -12235,7 +12266,7 @@
       <c r="BM170" s="1"/>
       <c r="BN170" s="1"/>
     </row>
-    <row r="171" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A171" s="1"/>
       <c r="B171" s="1"/>
       <c r="C171" s="1"/>
@@ -12303,7 +12334,7 @@
       <c r="BM171" s="1"/>
       <c r="BN171" s="1"/>
     </row>
-    <row r="172" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A172" s="1"/>
       <c r="B172" s="1"/>
       <c r="C172" s="1"/>
@@ -12371,7 +12402,7 @@
       <c r="BM172" s="1"/>
       <c r="BN172" s="1"/>
     </row>
-    <row r="173" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A173" s="1"/>
       <c r="B173" s="1"/>
       <c r="C173" s="1"/>
@@ -12439,7 +12470,7 @@
       <c r="BM173" s="1"/>
       <c r="BN173" s="1"/>
     </row>
-    <row r="174" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A174" s="1"/>
       <c r="B174" s="1"/>
       <c r="C174" s="1"/>
@@ -12507,7 +12538,7 @@
       <c r="BM174" s="1"/>
       <c r="BN174" s="1"/>
     </row>
-    <row r="175" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A175" s="1"/>
       <c r="B175" s="1"/>
       <c r="C175" s="1"/>
@@ -12575,7 +12606,7 @@
       <c r="BM175" s="1"/>
       <c r="BN175" s="1"/>
     </row>
-    <row r="176" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A176" s="1"/>
       <c r="B176" s="1"/>
       <c r="C176" s="1"/>
@@ -12643,7 +12674,7 @@
       <c r="BM176" s="1"/>
       <c r="BN176" s="1"/>
     </row>
-    <row r="177" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A177" s="1"/>
       <c r="B177" s="1"/>
       <c r="C177" s="1"/>
@@ -12711,7 +12742,7 @@
       <c r="BM177" s="1"/>
       <c r="BN177" s="1"/>
     </row>
-    <row r="178" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A178" s="1"/>
       <c r="B178" s="1"/>
       <c r="C178" s="1"/>
@@ -12779,7 +12810,7 @@
       <c r="BM178" s="1"/>
       <c r="BN178" s="1"/>
     </row>
-    <row r="179" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A179" s="1"/>
       <c r="B179" s="1"/>
       <c r="C179" s="1"/>
@@ -12847,7 +12878,7 @@
       <c r="BM179" s="1"/>
       <c r="BN179" s="1"/>
     </row>
-    <row r="180" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A180" s="1"/>
       <c r="B180" s="1"/>
       <c r="C180" s="1"/>
@@ -12915,7 +12946,7 @@
       <c r="BM180" s="1"/>
       <c r="BN180" s="1"/>
     </row>
-    <row r="181" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A181" s="1"/>
       <c r="B181" s="1"/>
       <c r="C181" s="1"/>
@@ -12983,7 +13014,7 @@
       <c r="BM181" s="1"/>
       <c r="BN181" s="1"/>
     </row>
-    <row r="182" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A182" s="1"/>
       <c r="B182" s="1"/>
       <c r="C182" s="1"/>
@@ -13051,7 +13082,7 @@
       <c r="BM182" s="1"/>
       <c r="BN182" s="1"/>
     </row>
-    <row r="183" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A183" s="1"/>
       <c r="B183" s="1"/>
       <c r="C183" s="1"/>
@@ -13119,7 +13150,7 @@
       <c r="BM183" s="1"/>
       <c r="BN183" s="1"/>
     </row>
-    <row r="184" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A184" s="1"/>
       <c r="B184" s="1"/>
       <c r="C184" s="1"/>
@@ -13187,7 +13218,7 @@
       <c r="BM184" s="1"/>
       <c r="BN184" s="1"/>
     </row>
-    <row r="185" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A185" s="1"/>
       <c r="B185" s="1"/>
       <c r="C185" s="1"/>
@@ -13255,7 +13286,7 @@
       <c r="BM185" s="1"/>
       <c r="BN185" s="1"/>
     </row>
-    <row r="186" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A186" s="1"/>
       <c r="B186" s="1"/>
       <c r="C186" s="1"/>
@@ -13323,7 +13354,7 @@
       <c r="BM186" s="1"/>
       <c r="BN186" s="1"/>
     </row>
-    <row r="187" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A187" s="1"/>
       <c r="B187" s="1"/>
       <c r="C187" s="1"/>
@@ -13391,7 +13422,7 @@
       <c r="BM187" s="1"/>
       <c r="BN187" s="1"/>
     </row>
-    <row r="188" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A188" s="1"/>
       <c r="B188" s="1"/>
       <c r="C188" s="1"/>
@@ -13459,7 +13490,7 @@
       <c r="BM188" s="1"/>
       <c r="BN188" s="1"/>
     </row>
-    <row r="189" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A189" s="1"/>
       <c r="B189" s="1"/>
       <c r="C189" s="1"/>
@@ -13527,7 +13558,7 @@
       <c r="BM189" s="1"/>
       <c r="BN189" s="1"/>
     </row>
-    <row r="190" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A190" s="1"/>
       <c r="B190" s="1"/>
       <c r="C190" s="1"/>
@@ -13595,7 +13626,7 @@
       <c r="BM190" s="1"/>
       <c r="BN190" s="1"/>
     </row>
-    <row r="191" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A191" s="1"/>
       <c r="B191" s="1"/>
       <c r="C191" s="1"/>
@@ -13663,7 +13694,7 @@
       <c r="BM191" s="1"/>
       <c r="BN191" s="1"/>
     </row>
-    <row r="192" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A192" s="1"/>
       <c r="B192" s="1"/>
       <c r="C192" s="1"/>
@@ -13731,7 +13762,7 @@
       <c r="BM192" s="1"/>
       <c r="BN192" s="1"/>
     </row>
-    <row r="193" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A193" s="1"/>
       <c r="B193" s="1"/>
       <c r="C193" s="1"/>
@@ -13799,7 +13830,7 @@
       <c r="BM193" s="1"/>
       <c r="BN193" s="1"/>
     </row>
-    <row r="194" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A194" s="1"/>
       <c r="B194" s="1"/>
       <c r="C194" s="1"/>
@@ -13867,7 +13898,7 @@
       <c r="BM194" s="1"/>
       <c r="BN194" s="1"/>
     </row>
-    <row r="195" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A195" s="1"/>
       <c r="B195" s="1"/>
       <c r="C195" s="1"/>
@@ -13935,7 +13966,7 @@
       <c r="BM195" s="1"/>
       <c r="BN195" s="1"/>
     </row>
-    <row r="196" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A196" s="1"/>
       <c r="B196" s="1"/>
       <c r="C196" s="1"/>
@@ -14003,7 +14034,7 @@
       <c r="BM196" s="1"/>
       <c r="BN196" s="1"/>
     </row>
-    <row r="197" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A197" s="1"/>
       <c r="B197" s="1"/>
       <c r="C197" s="1"/>
@@ -14071,7 +14102,7 @@
       <c r="BM197" s="1"/>
       <c r="BN197" s="1"/>
     </row>
-    <row r="198" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A198" s="1"/>
       <c r="B198" s="1"/>
       <c r="C198" s="1"/>
@@ -14139,7 +14170,7 @@
       <c r="BM198" s="1"/>
       <c r="BN198" s="1"/>
     </row>
-    <row r="199" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A199" s="1"/>
       <c r="B199" s="1"/>
       <c r="C199" s="1"/>
@@ -14207,7 +14238,7 @@
       <c r="BM199" s="1"/>
       <c r="BN199" s="1"/>
     </row>
-    <row r="200" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A200" s="1"/>
       <c r="B200" s="1"/>
       <c r="C200" s="1"/>
@@ -14275,7 +14306,7 @@
       <c r="BM200" s="1"/>
       <c r="BN200" s="1"/>
     </row>
-    <row r="201" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A201" s="1"/>
       <c r="B201" s="1"/>
       <c r="C201" s="1"/>
@@ -14343,7 +14374,7 @@
       <c r="BM201" s="1"/>
       <c r="BN201" s="1"/>
     </row>
-    <row r="202" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A202" s="1"/>
       <c r="B202" s="1"/>
       <c r="C202" s="1"/>
@@ -14411,7 +14442,7 @@
       <c r="BM202" s="1"/>
       <c r="BN202" s="1"/>
     </row>
-    <row r="203" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A203" s="1"/>
       <c r="B203" s="1"/>
       <c r="C203" s="1"/>
@@ -14479,7 +14510,7 @@
       <c r="BM203" s="1"/>
       <c r="BN203" s="1"/>
     </row>
-    <row r="204" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A204" s="1"/>
       <c r="B204" s="1"/>
       <c r="C204" s="1"/>
@@ -14547,7 +14578,7 @@
       <c r="BM204" s="1"/>
       <c r="BN204" s="1"/>
     </row>
-    <row r="205" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A205" s="1"/>
       <c r="B205" s="1"/>
       <c r="C205" s="1"/>
@@ -14615,7 +14646,7 @@
       <c r="BM205" s="1"/>
       <c r="BN205" s="1"/>
     </row>
-    <row r="206" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A206" s="1"/>
       <c r="B206" s="1"/>
       <c r="C206" s="1"/>
@@ -14683,7 +14714,7 @@
       <c r="BM206" s="1"/>
       <c r="BN206" s="1"/>
     </row>
-    <row r="207" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A207" s="1"/>
       <c r="B207" s="1"/>
       <c r="C207" s="1"/>
@@ -14751,7 +14782,7 @@
       <c r="BM207" s="1"/>
       <c r="BN207" s="1"/>
     </row>
-    <row r="208" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A208" s="1"/>
       <c r="B208" s="1"/>
       <c r="C208" s="1"/>
@@ -14819,7 +14850,7 @@
       <c r="BM208" s="1"/>
       <c r="BN208" s="1"/>
     </row>
-    <row r="209" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A209" s="1"/>
       <c r="B209" s="1"/>
       <c r="C209" s="1"/>
@@ -14887,7 +14918,7 @@
       <c r="BM209" s="1"/>
       <c r="BN209" s="1"/>
     </row>
-    <row r="210" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A210" s="1"/>
       <c r="B210" s="1"/>
       <c r="C210" s="1"/>
@@ -14955,7 +14986,7 @@
       <c r="BM210" s="1"/>
       <c r="BN210" s="1"/>
     </row>
-    <row r="211" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A211" s="1"/>
       <c r="B211" s="1"/>
       <c r="C211" s="1"/>
@@ -15023,7 +15054,7 @@
       <c r="BM211" s="1"/>
       <c r="BN211" s="1"/>
     </row>
-    <row r="212" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A212" s="1"/>
       <c r="B212" s="1"/>
       <c r="C212" s="1"/>
@@ -15091,7 +15122,7 @@
       <c r="BM212" s="1"/>
       <c r="BN212" s="1"/>
     </row>
-    <row r="213" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A213" s="1"/>
       <c r="B213" s="1"/>
       <c r="C213" s="1"/>
@@ -15159,7 +15190,7 @@
       <c r="BM213" s="1"/>
       <c r="BN213" s="1"/>
     </row>
-    <row r="214" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A214" s="1"/>
       <c r="B214" s="1"/>
       <c r="C214" s="1"/>
@@ -15227,7 +15258,7 @@
       <c r="BM214" s="1"/>
       <c r="BN214" s="1"/>
     </row>
-    <row r="215" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A215" s="1"/>
       <c r="B215" s="1"/>
       <c r="C215" s="1"/>
@@ -15295,7 +15326,7 @@
       <c r="BM215" s="1"/>
       <c r="BN215" s="1"/>
     </row>
-    <row r="216" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A216" s="1"/>
       <c r="B216" s="1"/>
       <c r="C216" s="1"/>
@@ -15363,7 +15394,7 @@
       <c r="BM216" s="1"/>
       <c r="BN216" s="1"/>
     </row>
-    <row r="217" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A217" s="1"/>
       <c r="B217" s="1"/>
       <c r="C217" s="1"/>
@@ -15431,7 +15462,7 @@
       <c r="BM217" s="1"/>
       <c r="BN217" s="1"/>
     </row>
-    <row r="218" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A218" s="1"/>
       <c r="B218" s="1"/>
       <c r="C218" s="1"/>
@@ -15499,7 +15530,7 @@
       <c r="BM218" s="1"/>
       <c r="BN218" s="1"/>
     </row>
-    <row r="219" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A219" s="1"/>
       <c r="B219" s="1"/>
       <c r="C219" s="1"/>
@@ -15567,7 +15598,7 @@
       <c r="BM219" s="1"/>
       <c r="BN219" s="1"/>
     </row>
-    <row r="220" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A220" s="1"/>
       <c r="B220" s="1"/>
       <c r="C220" s="1"/>
@@ -15635,7 +15666,7 @@
       <c r="BM220" s="1"/>
       <c r="BN220" s="1"/>
     </row>
-    <row r="221" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A221" s="1"/>
       <c r="B221" s="1"/>
       <c r="C221" s="1"/>
@@ -15703,7 +15734,7 @@
       <c r="BM221" s="1"/>
       <c r="BN221" s="1"/>
     </row>
-    <row r="222" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A222" s="1"/>
       <c r="B222" s="1"/>
       <c r="C222" s="1"/>
@@ -15771,7 +15802,7 @@
       <c r="BM222" s="1"/>
       <c r="BN222" s="1"/>
     </row>
-    <row r="223" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A223" s="1"/>
       <c r="B223" s="1"/>
       <c r="C223" s="1"/>
@@ -15839,7 +15870,7 @@
       <c r="BM223" s="1"/>
       <c r="BN223" s="1"/>
     </row>
-    <row r="224" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A224" s="1"/>
       <c r="B224" s="1"/>
       <c r="C224" s="1"/>
@@ -15907,7 +15938,7 @@
       <c r="BM224" s="1"/>
       <c r="BN224" s="1"/>
     </row>
-    <row r="225" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A225" s="1"/>
       <c r="B225" s="1"/>
       <c r="C225" s="1"/>
@@ -15975,7 +16006,7 @@
       <c r="BM225" s="1"/>
       <c r="BN225" s="1"/>
     </row>
-    <row r="226" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A226" s="1"/>
       <c r="B226" s="1"/>
       <c r="C226" s="1"/>
@@ -16043,7 +16074,7 @@
       <c r="BM226" s="1"/>
       <c r="BN226" s="1"/>
     </row>
-    <row r="227" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A227" s="1"/>
       <c r="B227" s="1"/>
       <c r="C227" s="1"/>
@@ -16111,7 +16142,7 @@
       <c r="BM227" s="1"/>
       <c r="BN227" s="1"/>
     </row>
-    <row r="228" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A228" s="1"/>
       <c r="B228" s="1"/>
       <c r="C228" s="1"/>
@@ -16179,7 +16210,7 @@
       <c r="BM228" s="1"/>
       <c r="BN228" s="1"/>
     </row>
-    <row r="229" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A229" s="1"/>
       <c r="B229" s="1"/>
       <c r="C229" s="1"/>
@@ -16247,7 +16278,7 @@
       <c r="BM229" s="1"/>
       <c r="BN229" s="1"/>
     </row>
-    <row r="230" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A230" s="1"/>
       <c r="B230" s="1"/>
       <c r="C230" s="1"/>
@@ -16315,7 +16346,7 @@
       <c r="BM230" s="1"/>
       <c r="BN230" s="1"/>
     </row>
-    <row r="231" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A231" s="1"/>
       <c r="B231" s="1"/>
       <c r="C231" s="1"/>
@@ -16383,7 +16414,7 @@
       <c r="BM231" s="1"/>
       <c r="BN231" s="1"/>
     </row>
-    <row r="232" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A232" s="1"/>
       <c r="B232" s="1"/>
       <c r="C232" s="1"/>
@@ -16451,7 +16482,7 @@
       <c r="BM232" s="1"/>
       <c r="BN232" s="1"/>
     </row>
-    <row r="233" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A233" s="1"/>
       <c r="B233" s="1"/>
       <c r="C233" s="1"/>
@@ -16519,7 +16550,7 @@
       <c r="BM233" s="1"/>
       <c r="BN233" s="1"/>
     </row>
-    <row r="234" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A234" s="1"/>
       <c r="B234" s="1"/>
       <c r="C234" s="1"/>
@@ -16587,7 +16618,7 @@
       <c r="BM234" s="1"/>
       <c r="BN234" s="1"/>
     </row>
-    <row r="235" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A235" s="1"/>
       <c r="B235" s="1"/>
       <c r="C235" s="1"/>
@@ -16655,7 +16686,7 @@
       <c r="BM235" s="1"/>
       <c r="BN235" s="1"/>
     </row>
-    <row r="236" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A236" s="1"/>
       <c r="B236" s="1"/>
       <c r="C236" s="1"/>
@@ -16723,7 +16754,7 @@
       <c r="BM236" s="1"/>
       <c r="BN236" s="1"/>
     </row>
-    <row r="237" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A237" s="1"/>
       <c r="B237" s="1"/>
       <c r="C237" s="1"/>
@@ -16791,7 +16822,7 @@
       <c r="BM237" s="1"/>
       <c r="BN237" s="1"/>
     </row>
-    <row r="238" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A238" s="1"/>
       <c r="B238" s="1"/>
       <c r="C238" s="1"/>
@@ -16859,7 +16890,7 @@
       <c r="BM238" s="1"/>
       <c r="BN238" s="1"/>
     </row>
-    <row r="239" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A239" s="1"/>
       <c r="B239" s="1"/>
       <c r="C239" s="1"/>
@@ -16927,7 +16958,7 @@
       <c r="BM239" s="1"/>
       <c r="BN239" s="1"/>
     </row>
-    <row r="240" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A240" s="1"/>
       <c r="B240" s="1"/>
       <c r="C240" s="1"/>
@@ -16995,7 +17026,7 @@
       <c r="BM240" s="1"/>
       <c r="BN240" s="1"/>
     </row>
-    <row r="241" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A241" s="1"/>
       <c r="B241" s="1"/>
       <c r="C241" s="1"/>
@@ -17063,7 +17094,7 @@
       <c r="BM241" s="1"/>
       <c r="BN241" s="1"/>
     </row>
-    <row r="242" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A242" s="1"/>
       <c r="B242" s="1"/>
       <c r="C242" s="1"/>
@@ -17131,7 +17162,7 @@
       <c r="BM242" s="1"/>
       <c r="BN242" s="1"/>
     </row>
-    <row r="243" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A243" s="1"/>
       <c r="B243" s="1"/>
       <c r="C243" s="1"/>
@@ -17199,7 +17230,7 @@
       <c r="BM243" s="1"/>
       <c r="BN243" s="1"/>
     </row>
-    <row r="244" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A244" s="1"/>
       <c r="B244" s="1"/>
       <c r="C244" s="1"/>
@@ -17267,7 +17298,7 @@
       <c r="BM244" s="1"/>
       <c r="BN244" s="1"/>
     </row>
-    <row r="245" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A245" s="1"/>
       <c r="B245" s="1"/>
       <c r="C245" s="1"/>
@@ -17335,7 +17366,7 @@
       <c r="BM245" s="1"/>
       <c r="BN245" s="1"/>
     </row>
-    <row r="246" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A246" s="1"/>
       <c r="B246" s="1"/>
       <c r="C246" s="1"/>
@@ -17403,7 +17434,7 @@
       <c r="BM246" s="1"/>
       <c r="BN246" s="1"/>
     </row>
-    <row r="247" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A247" s="1"/>
       <c r="B247" s="1"/>
       <c r="C247" s="1"/>
@@ -17471,7 +17502,7 @@
       <c r="BM247" s="1"/>
       <c r="BN247" s="1"/>
     </row>
-    <row r="248" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A248" s="1"/>
       <c r="B248" s="1"/>
       <c r="C248" s="1"/>
@@ -17539,7 +17570,7 @@
       <c r="BM248" s="1"/>
       <c r="BN248" s="1"/>
     </row>
-    <row r="249" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A249" s="1"/>
       <c r="B249" s="1"/>
       <c r="C249" s="1"/>
@@ -17607,7 +17638,7 @@
       <c r="BM249" s="1"/>
       <c r="BN249" s="1"/>
     </row>
-    <row r="250" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A250" s="1"/>
       <c r="B250" s="1"/>
       <c r="C250" s="1"/>
@@ -17675,7 +17706,7 @@
       <c r="BM250" s="1"/>
       <c r="BN250" s="1"/>
     </row>
-    <row r="251" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A251" s="1"/>
       <c r="B251" s="1"/>
       <c r="C251" s="1"/>
@@ -17743,7 +17774,7 @@
       <c r="BM251" s="1"/>
       <c r="BN251" s="1"/>
     </row>
-    <row r="252" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A252" s="1"/>
       <c r="B252" s="1"/>
       <c r="C252" s="1"/>
@@ -17811,7 +17842,7 @@
       <c r="BM252" s="1"/>
       <c r="BN252" s="1"/>
     </row>
-    <row r="253" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A253" s="1"/>
       <c r="B253" s="1"/>
       <c r="C253" s="1"/>
@@ -17879,7 +17910,7 @@
       <c r="BM253" s="1"/>
       <c r="BN253" s="1"/>
     </row>
-    <row r="254" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A254" s="1"/>
       <c r="B254" s="1"/>
       <c r="C254" s="1"/>
@@ -17947,7 +17978,7 @@
       <c r="BM254" s="1"/>
       <c r="BN254" s="1"/>
     </row>
-    <row r="255" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A255" s="1"/>
       <c r="B255" s="1"/>
       <c r="C255" s="1"/>
@@ -18015,7 +18046,7 @@
       <c r="BM255" s="1"/>
       <c r="BN255" s="1"/>
     </row>
-    <row r="256" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A256" s="1"/>
       <c r="B256" s="1"/>
       <c r="C256" s="1"/>
@@ -18083,7 +18114,7 @@
       <c r="BM256" s="1"/>
       <c r="BN256" s="1"/>
     </row>
-    <row r="257" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A257" s="1"/>
       <c r="B257" s="1"/>
       <c r="C257" s="1"/>
@@ -18151,7 +18182,7 @@
       <c r="BM257" s="1"/>
       <c r="BN257" s="1"/>
     </row>
-    <row r="258" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A258" s="1"/>
       <c r="B258" s="1"/>
       <c r="C258" s="1"/>
@@ -18219,7 +18250,7 @@
       <c r="BM258" s="1"/>
       <c r="BN258" s="1"/>
     </row>
-    <row r="259" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A259" s="1"/>
       <c r="B259" s="1"/>
       <c r="C259" s="1"/>
@@ -18287,7 +18318,7 @@
       <c r="BM259" s="1"/>
       <c r="BN259" s="1"/>
     </row>
-    <row r="260" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A260" s="1"/>
       <c r="B260" s="1"/>
       <c r="C260" s="1"/>
@@ -18355,7 +18386,7 @@
       <c r="BM260" s="1"/>
       <c r="BN260" s="1"/>
     </row>
-    <row r="261" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A261" s="1"/>
       <c r="B261" s="1"/>
       <c r="C261" s="1"/>
@@ -18423,7 +18454,7 @@
       <c r="BM261" s="1"/>
       <c r="BN261" s="1"/>
     </row>
-    <row r="262" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A262" s="1"/>
       <c r="B262" s="1"/>
       <c r="C262" s="1"/>
@@ -18491,7 +18522,7 @@
       <c r="BM262" s="1"/>
       <c r="BN262" s="1"/>
     </row>
-    <row r="263" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A263" s="1"/>
       <c r="B263" s="1"/>
       <c r="C263" s="1"/>
@@ -18559,7 +18590,7 @@
       <c r="BM263" s="1"/>
       <c r="BN263" s="1"/>
     </row>
-    <row r="264" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A264" s="1"/>
       <c r="B264" s="1"/>
       <c r="C264" s="1"/>
@@ -18627,7 +18658,7 @@
       <c r="BM264" s="1"/>
       <c r="BN264" s="1"/>
     </row>
-    <row r="265" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:66" x14ac:dyDescent="0.5">
       <c r="A265" s="1"/>
       <c r="B265" s="1"/>
       <c r="C265" s="1"/>
@@ -18695,7 +18726,7 @@
       <c r="BM265" s="1"/>
       <c r="BN265" s="1"/>
     </row>
-    <row r="266" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:66" x14ac:dyDescent="0.5">
       <c r="H266" s="1"/>
       <c r="I266" s="1"/>
       <c r="J266" s="1"/>
@@ -18756,7 +18787,7 @@
       <c r="BM266" s="1"/>
       <c r="BN266" s="1"/>
     </row>
-    <row r="267" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:66" x14ac:dyDescent="0.5">
       <c r="H267" s="1"/>
       <c r="I267" s="1"/>
       <c r="J267" s="1"/>
@@ -18817,7 +18848,7 @@
       <c r="BM267" s="1"/>
       <c r="BN267" s="1"/>
     </row>
-    <row r="268" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:66" x14ac:dyDescent="0.5">
       <c r="H268" s="1"/>
       <c r="I268" s="1"/>
       <c r="J268" s="1"/>
@@ -18878,7 +18909,7 @@
       <c r="BM268" s="1"/>
       <c r="BN268" s="1"/>
     </row>
-    <row r="269" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:66" x14ac:dyDescent="0.5">
       <c r="H269" s="1"/>
       <c r="I269" s="1"/>
       <c r="J269" s="1"/>
@@ -18939,7 +18970,7 @@
       <c r="BM269" s="1"/>
       <c r="BN269" s="1"/>
     </row>
-    <row r="270" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:66" x14ac:dyDescent="0.5">
       <c r="H270" s="1"/>
       <c r="I270" s="1"/>
       <c r="J270" s="1"/>
@@ -19000,7 +19031,7 @@
       <c r="BM270" s="1"/>
       <c r="BN270" s="1"/>
     </row>
-    <row r="271" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:66" x14ac:dyDescent="0.5">
       <c r="H271" s="1"/>
       <c r="I271" s="1"/>
       <c r="J271" s="1"/>
@@ -19061,7 +19092,7 @@
       <c r="BM271" s="1"/>
       <c r="BN271" s="1"/>
     </row>
-    <row r="272" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:66" x14ac:dyDescent="0.5">
       <c r="H272" s="1"/>
       <c r="I272" s="1"/>
       <c r="J272" s="1"/>
@@ -19122,7 +19153,7 @@
       <c r="BM272" s="1"/>
       <c r="BN272" s="1"/>
     </row>
-    <row r="273" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="273" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H273" s="1"/>
       <c r="I273" s="1"/>
       <c r="J273" s="1"/>
@@ -19183,7 +19214,7 @@
       <c r="BM273" s="1"/>
       <c r="BN273" s="1"/>
     </row>
-    <row r="274" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="274" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H274" s="1"/>
       <c r="I274" s="1"/>
       <c r="J274" s="1"/>
@@ -19244,7 +19275,7 @@
       <c r="BM274" s="1"/>
       <c r="BN274" s="1"/>
     </row>
-    <row r="275" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="275" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H275" s="1"/>
       <c r="I275" s="1"/>
       <c r="J275" s="1"/>
@@ -19305,7 +19336,7 @@
       <c r="BM275" s="1"/>
       <c r="BN275" s="1"/>
     </row>
-    <row r="276" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="276" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H276" s="1"/>
       <c r="I276" s="1"/>
       <c r="J276" s="1"/>
@@ -19366,7 +19397,7 @@
       <c r="BM276" s="1"/>
       <c r="BN276" s="1"/>
     </row>
-    <row r="277" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="277" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H277" s="1"/>
       <c r="I277" s="1"/>
       <c r="J277" s="1"/>
@@ -19427,7 +19458,7 @@
       <c r="BM277" s="1"/>
       <c r="BN277" s="1"/>
     </row>
-    <row r="278" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="278" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H278" s="1"/>
       <c r="I278" s="1"/>
       <c r="J278" s="1"/>
@@ -19488,7 +19519,7 @@
       <c r="BM278" s="1"/>
       <c r="BN278" s="1"/>
     </row>
-    <row r="279" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="279" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H279" s="1"/>
       <c r="I279" s="1"/>
       <c r="J279" s="1"/>
@@ -19549,7 +19580,7 @@
       <c r="BM279" s="1"/>
       <c r="BN279" s="1"/>
     </row>
-    <row r="280" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="280" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H280" s="1"/>
       <c r="I280" s="1"/>
       <c r="J280" s="1"/>
@@ -19610,7 +19641,7 @@
       <c r="BM280" s="1"/>
       <c r="BN280" s="1"/>
     </row>
-    <row r="281" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="281" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H281" s="1"/>
       <c r="I281" s="1"/>
       <c r="J281" s="1"/>
@@ -19671,7 +19702,7 @@
       <c r="BM281" s="1"/>
       <c r="BN281" s="1"/>
     </row>
-    <row r="282" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="282" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H282" s="1"/>
       <c r="I282" s="1"/>
       <c r="J282" s="1"/>
@@ -19732,7 +19763,7 @@
       <c r="BM282" s="1"/>
       <c r="BN282" s="1"/>
     </row>
-    <row r="283" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="283" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H283" s="1"/>
       <c r="I283" s="1"/>
       <c r="J283" s="1"/>
@@ -19793,7 +19824,7 @@
       <c r="BM283" s="1"/>
       <c r="BN283" s="1"/>
     </row>
-    <row r="284" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="284" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H284" s="1"/>
       <c r="I284" s="1"/>
       <c r="J284" s="1"/>
@@ -19854,7 +19885,7 @@
       <c r="BM284" s="1"/>
       <c r="BN284" s="1"/>
     </row>
-    <row r="285" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="285" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H285" s="1"/>
       <c r="I285" s="1"/>
       <c r="J285" s="1"/>
@@ -19915,7 +19946,7 @@
       <c r="BM285" s="1"/>
       <c r="BN285" s="1"/>
     </row>
-    <row r="286" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="286" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H286" s="1"/>
       <c r="I286" s="1"/>
       <c r="J286" s="1"/>
@@ -19976,7 +20007,7 @@
       <c r="BM286" s="1"/>
       <c r="BN286" s="1"/>
     </row>
-    <row r="287" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="287" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H287" s="1"/>
       <c r="I287" s="1"/>
       <c r="J287" s="1"/>
@@ -20037,7 +20068,7 @@
       <c r="BM287" s="1"/>
       <c r="BN287" s="1"/>
     </row>
-    <row r="288" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="288" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H288" s="1"/>
       <c r="I288" s="1"/>
       <c r="J288" s="1"/>
@@ -20098,7 +20129,7 @@
       <c r="BM288" s="1"/>
       <c r="BN288" s="1"/>
     </row>
-    <row r="289" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="289" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H289" s="1"/>
       <c r="I289" s="1"/>
       <c r="J289" s="1"/>
@@ -20159,7 +20190,7 @@
       <c r="BM289" s="1"/>
       <c r="BN289" s="1"/>
     </row>
-    <row r="290" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="290" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H290" s="1"/>
       <c r="I290" s="1"/>
       <c r="J290" s="1"/>
@@ -20220,7 +20251,7 @@
       <c r="BM290" s="1"/>
       <c r="BN290" s="1"/>
     </row>
-    <row r="291" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="291" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H291" s="1"/>
       <c r="I291" s="1"/>
       <c r="J291" s="1"/>
@@ -20281,7 +20312,7 @@
       <c r="BM291" s="1"/>
       <c r="BN291" s="1"/>
     </row>
-    <row r="292" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="292" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H292" s="1"/>
       <c r="I292" s="1"/>
       <c r="J292" s="1"/>
@@ -20342,7 +20373,7 @@
       <c r="BM292" s="1"/>
       <c r="BN292" s="1"/>
     </row>
-    <row r="293" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="293" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H293" s="1"/>
       <c r="I293" s="1"/>
       <c r="J293" s="1"/>
@@ -20403,7 +20434,7 @@
       <c r="BM293" s="1"/>
       <c r="BN293" s="1"/>
     </row>
-    <row r="294" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="294" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H294" s="1"/>
       <c r="I294" s="1"/>
       <c r="J294" s="1"/>
@@ -20464,7 +20495,7 @@
       <c r="BM294" s="1"/>
       <c r="BN294" s="1"/>
     </row>
-    <row r="295" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="295" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H295" s="1"/>
       <c r="I295" s="1"/>
       <c r="J295" s="1"/>
@@ -20525,7 +20556,7 @@
       <c r="BM295" s="1"/>
       <c r="BN295" s="1"/>
     </row>
-    <row r="296" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="296" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H296" s="1"/>
       <c r="I296" s="1"/>
       <c r="J296" s="1"/>
@@ -20586,7 +20617,7 @@
       <c r="BM296" s="1"/>
       <c r="BN296" s="1"/>
     </row>
-    <row r="297" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="297" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H297" s="1"/>
       <c r="I297" s="1"/>
       <c r="J297" s="1"/>
@@ -20647,7 +20678,7 @@
       <c r="BM297" s="1"/>
       <c r="BN297" s="1"/>
     </row>
-    <row r="298" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="298" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H298" s="1"/>
       <c r="I298" s="1"/>
       <c r="J298" s="1"/>
@@ -20708,7 +20739,7 @@
       <c r="BM298" s="1"/>
       <c r="BN298" s="1"/>
     </row>
-    <row r="299" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="299" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H299" s="1"/>
       <c r="I299" s="1"/>
       <c r="J299" s="1"/>
@@ -20769,7 +20800,7 @@
       <c r="BM299" s="1"/>
       <c r="BN299" s="1"/>
     </row>
-    <row r="300" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="300" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H300" s="1"/>
       <c r="I300" s="1"/>
       <c r="J300" s="1"/>
@@ -20830,7 +20861,7 @@
       <c r="BM300" s="1"/>
       <c r="BN300" s="1"/>
     </row>
-    <row r="301" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="301" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H301" s="1"/>
       <c r="I301" s="1"/>
       <c r="J301" s="1"/>
@@ -20891,7 +20922,7 @@
       <c r="BM301" s="1"/>
       <c r="BN301" s="1"/>
     </row>
-    <row r="302" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="302" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H302" s="1"/>
       <c r="I302" s="1"/>
       <c r="J302" s="1"/>
@@ -20952,7 +20983,7 @@
       <c r="BM302" s="1"/>
       <c r="BN302" s="1"/>
     </row>
-    <row r="303" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="303" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H303" s="1"/>
       <c r="I303" s="1"/>
       <c r="J303" s="1"/>
@@ -21013,7 +21044,7 @@
       <c r="BM303" s="1"/>
       <c r="BN303" s="1"/>
     </row>
-    <row r="304" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="304" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H304" s="1"/>
       <c r="I304" s="1"/>
       <c r="J304" s="1"/>
@@ -21074,7 +21105,7 @@
       <c r="BM304" s="1"/>
       <c r="BN304" s="1"/>
     </row>
-    <row r="305" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="305" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H305" s="1"/>
       <c r="I305" s="1"/>
       <c r="J305" s="1"/>
@@ -21135,7 +21166,7 @@
       <c r="BM305" s="1"/>
       <c r="BN305" s="1"/>
     </row>
-    <row r="306" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="306" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H306" s="1"/>
       <c r="I306" s="1"/>
       <c r="J306" s="1"/>
@@ -21196,7 +21227,7 @@
       <c r="BM306" s="1"/>
       <c r="BN306" s="1"/>
     </row>
-    <row r="307" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="307" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H307" s="1"/>
       <c r="I307" s="1"/>
       <c r="J307" s="1"/>
@@ -21257,7 +21288,7 @@
       <c r="BM307" s="1"/>
       <c r="BN307" s="1"/>
     </row>
-    <row r="308" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="308" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H308" s="1"/>
       <c r="I308" s="1"/>
       <c r="J308" s="1"/>
@@ -21318,7 +21349,7 @@
       <c r="BM308" s="1"/>
       <c r="BN308" s="1"/>
     </row>
-    <row r="309" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="309" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H309" s="1"/>
       <c r="I309" s="1"/>
       <c r="J309" s="1"/>
@@ -21379,7 +21410,7 @@
       <c r="BM309" s="1"/>
       <c r="BN309" s="1"/>
     </row>
-    <row r="310" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="310" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H310" s="1"/>
       <c r="I310" s="1"/>
       <c r="J310" s="1"/>
@@ -21440,7 +21471,7 @@
       <c r="BM310" s="1"/>
       <c r="BN310" s="1"/>
     </row>
-    <row r="311" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="311" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H311" s="1"/>
       <c r="I311" s="1"/>
       <c r="J311" s="1"/>
@@ -21501,7 +21532,7 @@
       <c r="BM311" s="1"/>
       <c r="BN311" s="1"/>
     </row>
-    <row r="312" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="312" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H312" s="1"/>
       <c r="I312" s="1"/>
       <c r="J312" s="1"/>
@@ -21562,7 +21593,7 @@
       <c r="BM312" s="1"/>
       <c r="BN312" s="1"/>
     </row>
-    <row r="313" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="313" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H313" s="1"/>
       <c r="I313" s="1"/>
       <c r="J313" s="1"/>
@@ -21623,7 +21654,7 @@
       <c r="BM313" s="1"/>
       <c r="BN313" s="1"/>
     </row>
-    <row r="314" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="314" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H314" s="1"/>
       <c r="I314" s="1"/>
       <c r="J314" s="1"/>
@@ -21684,7 +21715,7 @@
       <c r="BM314" s="1"/>
       <c r="BN314" s="1"/>
     </row>
-    <row r="315" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="315" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H315" s="1"/>
       <c r="I315" s="1"/>
       <c r="J315" s="1"/>
@@ -21745,7 +21776,7 @@
       <c r="BM315" s="1"/>
       <c r="BN315" s="1"/>
     </row>
-    <row r="316" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="316" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H316" s="1"/>
       <c r="I316" s="1"/>
       <c r="J316" s="1"/>
@@ -21806,7 +21837,7 @@
       <c r="BM316" s="1"/>
       <c r="BN316" s="1"/>
     </row>
-    <row r="317" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="317" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H317" s="1"/>
       <c r="I317" s="1"/>
       <c r="J317" s="1"/>
@@ -21867,7 +21898,7 @@
       <c r="BM317" s="1"/>
       <c r="BN317" s="1"/>
     </row>
-    <row r="318" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="318" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H318" s="1"/>
       <c r="I318" s="1"/>
       <c r="J318" s="1"/>
@@ -21928,7 +21959,7 @@
       <c r="BM318" s="1"/>
       <c r="BN318" s="1"/>
     </row>
-    <row r="319" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="319" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H319" s="1"/>
       <c r="I319" s="1"/>
       <c r="J319" s="1"/>
@@ -21989,7 +22020,7 @@
       <c r="BM319" s="1"/>
       <c r="BN319" s="1"/>
     </row>
-    <row r="320" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="320" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H320" s="1"/>
       <c r="I320" s="1"/>
       <c r="J320" s="1"/>
@@ -22050,7 +22081,7 @@
       <c r="BM320" s="1"/>
       <c r="BN320" s="1"/>
     </row>
-    <row r="321" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="321" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H321" s="1"/>
       <c r="I321" s="1"/>
       <c r="J321" s="1"/>
@@ -22111,7 +22142,7 @@
       <c r="BM321" s="1"/>
       <c r="BN321" s="1"/>
     </row>
-    <row r="322" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="322" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H322" s="1"/>
       <c r="I322" s="1"/>
       <c r="J322" s="1"/>
@@ -22172,7 +22203,7 @@
       <c r="BM322" s="1"/>
       <c r="BN322" s="1"/>
     </row>
-    <row r="323" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="323" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H323" s="1"/>
       <c r="I323" s="1"/>
       <c r="J323" s="1"/>
@@ -22233,7 +22264,7 @@
       <c r="BM323" s="1"/>
       <c r="BN323" s="1"/>
     </row>
-    <row r="324" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="324" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H324" s="1"/>
       <c r="I324" s="1"/>
       <c r="J324" s="1"/>
@@ -22294,7 +22325,7 @@
       <c r="BM324" s="1"/>
       <c r="BN324" s="1"/>
     </row>
-    <row r="325" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="325" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H325" s="1"/>
       <c r="I325" s="1"/>
       <c r="J325" s="1"/>
@@ -22355,7 +22386,7 @@
       <c r="BM325" s="1"/>
       <c r="BN325" s="1"/>
     </row>
-    <row r="326" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="326" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H326" s="1"/>
       <c r="I326" s="1"/>
       <c r="J326" s="1"/>
@@ -22416,7 +22447,7 @@
       <c r="BM326" s="1"/>
       <c r="BN326" s="1"/>
     </row>
-    <row r="327" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="327" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H327" s="1"/>
       <c r="I327" s="1"/>
       <c r="J327" s="1"/>
@@ -22477,7 +22508,7 @@
       <c r="BM327" s="1"/>
       <c r="BN327" s="1"/>
     </row>
-    <row r="328" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="328" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H328" s="1"/>
       <c r="I328" s="1"/>
       <c r="J328" s="1"/>
@@ -22538,7 +22569,7 @@
       <c r="BM328" s="1"/>
       <c r="BN328" s="1"/>
     </row>
-    <row r="329" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="329" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H329" s="1"/>
       <c r="I329" s="1"/>
       <c r="J329" s="1"/>
@@ -22599,7 +22630,7 @@
       <c r="BM329" s="1"/>
       <c r="BN329" s="1"/>
     </row>
-    <row r="330" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="330" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H330" s="1"/>
       <c r="I330" s="1"/>
       <c r="J330" s="1"/>
@@ -22660,7 +22691,7 @@
       <c r="BM330" s="1"/>
       <c r="BN330" s="1"/>
     </row>
-    <row r="331" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="331" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H331" s="1"/>
       <c r="I331" s="1"/>
       <c r="J331" s="1"/>
@@ -22721,7 +22752,7 @@
       <c r="BM331" s="1"/>
       <c r="BN331" s="1"/>
     </row>
-    <row r="332" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="332" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H332" s="1"/>
       <c r="I332" s="1"/>
       <c r="J332" s="1"/>
@@ -22782,7 +22813,7 @@
       <c r="BM332" s="1"/>
       <c r="BN332" s="1"/>
     </row>
-    <row r="333" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="333" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H333" s="1"/>
       <c r="I333" s="1"/>
       <c r="J333" s="1"/>
@@ -22843,7 +22874,7 @@
       <c r="BM333" s="1"/>
       <c r="BN333" s="1"/>
     </row>
-    <row r="334" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="334" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H334" s="1"/>
       <c r="I334" s="1"/>
       <c r="J334" s="1"/>
@@ -22904,7 +22935,7 @@
       <c r="BM334" s="1"/>
       <c r="BN334" s="1"/>
     </row>
-    <row r="335" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="335" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H335" s="1"/>
       <c r="I335" s="1"/>
       <c r="J335" s="1"/>
@@ -22965,7 +22996,7 @@
       <c r="BM335" s="1"/>
       <c r="BN335" s="1"/>
     </row>
-    <row r="336" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="336" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H336" s="1"/>
       <c r="I336" s="1"/>
       <c r="J336" s="1"/>
@@ -23026,7 +23057,7 @@
       <c r="BM336" s="1"/>
       <c r="BN336" s="1"/>
     </row>
-    <row r="337" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="337" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H337" s="1"/>
       <c r="I337" s="1"/>
       <c r="J337" s="1"/>
@@ -23087,7 +23118,7 @@
       <c r="BM337" s="1"/>
       <c r="BN337" s="1"/>
     </row>
-    <row r="338" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="338" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H338" s="1"/>
       <c r="I338" s="1"/>
       <c r="J338" s="1"/>
@@ -23148,7 +23179,7 @@
       <c r="BM338" s="1"/>
       <c r="BN338" s="1"/>
     </row>
-    <row r="339" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="339" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H339" s="1"/>
       <c r="I339" s="1"/>
       <c r="J339" s="1"/>
@@ -23209,7 +23240,7 @@
       <c r="BM339" s="1"/>
       <c r="BN339" s="1"/>
     </row>
-    <row r="340" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="340" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H340" s="1"/>
       <c r="I340" s="1"/>
       <c r="J340" s="1"/>
@@ -23270,7 +23301,7 @@
       <c r="BM340" s="1"/>
       <c r="BN340" s="1"/>
     </row>
-    <row r="341" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="341" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H341" s="1"/>
       <c r="I341" s="1"/>
       <c r="J341" s="1"/>
@@ -23331,7 +23362,7 @@
       <c r="BM341" s="1"/>
       <c r="BN341" s="1"/>
     </row>
-    <row r="342" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="342" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H342" s="1"/>
       <c r="I342" s="1"/>
       <c r="J342" s="1"/>
@@ -23392,7 +23423,7 @@
       <c r="BM342" s="1"/>
       <c r="BN342" s="1"/>
     </row>
-    <row r="343" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="343" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H343" s="1"/>
       <c r="I343" s="1"/>
       <c r="J343" s="1"/>
@@ -23453,7 +23484,7 @@
       <c r="BM343" s="1"/>
       <c r="BN343" s="1"/>
     </row>
-    <row r="344" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="344" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H344" s="1"/>
       <c r="I344" s="1"/>
       <c r="J344" s="1"/>
@@ -23514,7 +23545,7 @@
       <c r="BM344" s="1"/>
       <c r="BN344" s="1"/>
     </row>
-    <row r="345" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="345" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H345" s="1"/>
       <c r="I345" s="1"/>
       <c r="J345" s="1"/>
@@ -23575,7 +23606,7 @@
       <c r="BM345" s="1"/>
       <c r="BN345" s="1"/>
     </row>
-    <row r="346" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="346" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H346" s="1"/>
       <c r="I346" s="1"/>
       <c r="J346" s="1"/>
@@ -23636,7 +23667,7 @@
       <c r="BM346" s="1"/>
       <c r="BN346" s="1"/>
     </row>
-    <row r="347" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="347" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H347" s="1"/>
       <c r="I347" s="1"/>
       <c r="J347" s="1"/>
@@ -23697,7 +23728,7 @@
       <c r="BM347" s="1"/>
       <c r="BN347" s="1"/>
     </row>
-    <row r="348" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="348" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H348" s="1"/>
       <c r="I348" s="1"/>
       <c r="J348" s="1"/>
@@ -23758,7 +23789,7 @@
       <c r="BM348" s="1"/>
       <c r="BN348" s="1"/>
     </row>
-    <row r="349" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="349" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H349" s="1"/>
       <c r="I349" s="1"/>
       <c r="J349" s="1"/>
@@ -23819,7 +23850,7 @@
       <c r="BM349" s="1"/>
       <c r="BN349" s="1"/>
     </row>
-    <row r="350" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="350" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H350" s="1"/>
       <c r="I350" s="1"/>
       <c r="J350" s="1"/>
@@ -23880,7 +23911,7 @@
       <c r="BM350" s="1"/>
       <c r="BN350" s="1"/>
     </row>
-    <row r="351" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="351" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H351" s="1"/>
       <c r="I351" s="1"/>
       <c r="J351" s="1"/>
@@ -23941,7 +23972,7 @@
       <c r="BM351" s="1"/>
       <c r="BN351" s="1"/>
     </row>
-    <row r="352" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="352" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H352" s="1"/>
       <c r="I352" s="1"/>
       <c r="J352" s="1"/>
@@ -24002,7 +24033,7 @@
       <c r="BM352" s="1"/>
       <c r="BN352" s="1"/>
     </row>
-    <row r="353" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="353" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H353" s="1"/>
       <c r="I353" s="1"/>
       <c r="J353" s="1"/>
@@ -24063,7 +24094,7 @@
       <c r="BM353" s="1"/>
       <c r="BN353" s="1"/>
     </row>
-    <row r="354" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="354" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H354" s="1"/>
       <c r="I354" s="1"/>
       <c r="J354" s="1"/>
@@ -24124,7 +24155,7 @@
       <c r="BM354" s="1"/>
       <c r="BN354" s="1"/>
     </row>
-    <row r="355" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="355" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H355" s="1"/>
       <c r="I355" s="1"/>
       <c r="J355" s="1"/>
@@ -24185,7 +24216,7 @@
       <c r="BM355" s="1"/>
       <c r="BN355" s="1"/>
     </row>
-    <row r="356" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="356" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H356" s="1"/>
       <c r="I356" s="1"/>
       <c r="J356" s="1"/>
@@ -24246,7 +24277,7 @@
       <c r="BM356" s="1"/>
       <c r="BN356" s="1"/>
     </row>
-    <row r="357" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="357" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H357" s="1"/>
       <c r="I357" s="1"/>
       <c r="J357" s="1"/>
@@ -24307,7 +24338,7 @@
       <c r="BM357" s="1"/>
       <c r="BN357" s="1"/>
     </row>
-    <row r="358" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="358" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H358" s="1"/>
       <c r="I358" s="1"/>
       <c r="J358" s="1"/>
@@ -24368,7 +24399,7 @@
       <c r="BM358" s="1"/>
       <c r="BN358" s="1"/>
     </row>
-    <row r="359" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="359" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H359" s="1"/>
       <c r="I359" s="1"/>
       <c r="J359" s="1"/>
@@ -24429,7 +24460,7 @@
       <c r="BM359" s="1"/>
       <c r="BN359" s="1"/>
     </row>
-    <row r="360" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="360" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H360" s="1"/>
       <c r="I360" s="1"/>
       <c r="J360" s="1"/>
@@ -24490,7 +24521,7 @@
       <c r="BM360" s="1"/>
       <c r="BN360" s="1"/>
     </row>
-    <row r="361" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="361" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H361" s="1"/>
       <c r="I361" s="1"/>
       <c r="J361" s="1"/>
@@ -24551,7 +24582,7 @@
       <c r="BM361" s="1"/>
       <c r="BN361" s="1"/>
     </row>
-    <row r="362" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="362" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H362" s="1"/>
       <c r="I362" s="1"/>
       <c r="J362" s="1"/>
@@ -24612,7 +24643,7 @@
       <c r="BM362" s="1"/>
       <c r="BN362" s="1"/>
     </row>
-    <row r="363" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="363" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H363" s="1"/>
       <c r="I363" s="1"/>
       <c r="J363" s="1"/>
@@ -24673,7 +24704,7 @@
       <c r="BM363" s="1"/>
       <c r="BN363" s="1"/>
     </row>
-    <row r="364" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="364" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H364" s="1"/>
       <c r="I364" s="1"/>
       <c r="J364" s="1"/>
@@ -24734,7 +24765,7 @@
       <c r="BM364" s="1"/>
       <c r="BN364" s="1"/>
     </row>
-    <row r="365" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="365" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H365" s="1"/>
       <c r="I365" s="1"/>
       <c r="J365" s="1"/>
@@ -24795,7 +24826,7 @@
       <c r="BM365" s="1"/>
       <c r="BN365" s="1"/>
     </row>
-    <row r="366" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="366" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H366" s="1"/>
       <c r="I366" s="1"/>
       <c r="J366" s="1"/>
@@ -24856,7 +24887,7 @@
       <c r="BM366" s="1"/>
       <c r="BN366" s="1"/>
     </row>
-    <row r="367" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="367" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H367" s="1"/>
       <c r="I367" s="1"/>
       <c r="J367" s="1"/>
@@ -24917,7 +24948,7 @@
       <c r="BM367" s="1"/>
       <c r="BN367" s="1"/>
     </row>
-    <row r="368" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="368" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H368" s="1"/>
       <c r="I368" s="1"/>
       <c r="J368" s="1"/>
@@ -24978,7 +25009,7 @@
       <c r="BM368" s="1"/>
       <c r="BN368" s="1"/>
     </row>
-    <row r="369" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="369" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H369" s="1"/>
       <c r="I369" s="1"/>
       <c r="J369" s="1"/>
@@ -25039,7 +25070,7 @@
       <c r="BM369" s="1"/>
       <c r="BN369" s="1"/>
     </row>
-    <row r="370" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="370" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H370" s="1"/>
       <c r="I370" s="1"/>
       <c r="J370" s="1"/>
@@ -25100,7 +25131,7 @@
       <c r="BM370" s="1"/>
       <c r="BN370" s="1"/>
     </row>
-    <row r="371" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="371" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H371" s="1"/>
       <c r="I371" s="1"/>
       <c r="J371" s="1"/>
@@ -25161,7 +25192,7 @@
       <c r="BM371" s="1"/>
       <c r="BN371" s="1"/>
     </row>
-    <row r="372" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="372" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H372" s="1"/>
       <c r="I372" s="1"/>
       <c r="J372" s="1"/>
@@ -25222,7 +25253,7 @@
       <c r="BM372" s="1"/>
       <c r="BN372" s="1"/>
     </row>
-    <row r="373" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="373" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H373" s="1"/>
       <c r="I373" s="1"/>
       <c r="J373" s="1"/>
@@ -25283,7 +25314,7 @@
       <c r="BM373" s="1"/>
       <c r="BN373" s="1"/>
     </row>
-    <row r="374" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="374" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H374" s="1"/>
       <c r="I374" s="1"/>
       <c r="J374" s="1"/>
@@ -25344,7 +25375,7 @@
       <c r="BM374" s="1"/>
       <c r="BN374" s="1"/>
     </row>
-    <row r="375" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="375" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H375" s="1"/>
       <c r="I375" s="1"/>
       <c r="J375" s="1"/>
@@ -25405,7 +25436,7 @@
       <c r="BM375" s="1"/>
       <c r="BN375" s="1"/>
     </row>
-    <row r="376" spans="8:66" x14ac:dyDescent="0.25">
+    <row r="376" spans="8:66" x14ac:dyDescent="0.5">
       <c r="H376" s="1"/>
       <c r="I376" s="1"/>
       <c r="J376" s="1"/>
@@ -25467,11 +25498,37 @@
       <c r="BN376" s="1"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B3:G26">
-    <cfRule type="expression" dxfId="0" priority="2">
+  <autoFilter ref="B2:G10" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:G10">
+      <sortCondition ref="E2:E10"/>
+    </sortState>
+  </autoFilter>
+  <conditionalFormatting sqref="B26:D26 F26:G26 B20:G25 B19:D19 F19:G19 B11:G18 B10:D10 F10:G10 B3:G9">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>$C3="Completed"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="E26">
+    <cfRule type="expression" dxfId="1" priority="4">
+      <formula>$C4="Completed"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E3">
+    <cfRule type="expression" dxfId="0" priority="6">
+      <formula>$C19="Completed"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:D26" xr:uid="{3950671C-D662-7A44-893B-6DD73468F32C}">
+      <formula1>"Tief,Mittel,Hoch"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C3:C26" xr:uid="{C89972C3-D511-5C48-978C-17F19E3F1C1B}">
+      <formula1>"To Do,Informieren,Planen,Entscheiden,Realisieren,Kontrollieren,Auswerten,Done"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3:E26" xr:uid="{8BC78E98-0B5D-4B64-A81C-ADA2AFBCF415}">
+      <formula1>"18.05.2026,25.05.2026,01.06.2026,08.06.2026"</formula1>
+    </dataValidation>
+  </dataValidations>
   <hyperlinks>
     <hyperlink ref="I29" r:id="rId1" display="Or, Click Here to Create a Project Budget Sheet in Smartsheet" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="J29" r:id="rId2" display="Or, Click Here to Create a Project Budget Sheet in Smartsheet" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
@@ -25483,24 +25540,8 @@
     <hyperlink ref="L30" r:id="rId8" display="Or, Click Here to Create a Project Budget Sheet in Smartsheet" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" verticalDpi="0"/>
+  <pageSetup orientation="portrait" r:id="rId9"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3950671C-D662-7A44-893B-6DD73468F32C}">
-          <x14:formula1>
-            <xm:f>'-Drop Down Keys-'!$D$3:$D$5</xm:f>
-          </x14:formula1>
-          <xm:sqref>D3:D26</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C89972C3-D511-5C48-978C-17F19E3F1C1B}">
-          <x14:formula1>
-            <xm:f>'-Drop Down Keys-'!$B$3:$B$6</xm:f>
-          </x14:formula1>
-          <xm:sqref>C3:C26</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
       <mx:PLV Mode="0" OnePage="0" WScale="0"/>
     </ext>
@@ -25511,121 +25552,121 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECDFC8D6-54EF-E94E-B38B-51BFD1BD45A3}">
   <dimension ref="B1:D19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="4.125" customWidth="1"/>
     <col min="2" max="2" width="19.375" customWidth="1"/>
     <col min="4" max="4" width="21.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" ht="57" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="7" t="s">
+    <row r="1" spans="2:4" ht="57" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B1" s="6" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="2:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="5" t="s">
+    <row r="2" spans="2:4" ht="30" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="6" t="s">
+      <c r="C2" s="2"/>
+      <c r="D2" s="5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="14" t="s">
+    <row r="3" spans="2:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B3" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="4" t="s">
-        <v>15</v>
+      <c r="C3" s="2"/>
+      <c r="D3" s="3" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="3" t="s">
-        <v>14</v>
+    <row r="4" spans="2:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B4" s="2" t="s">
+        <v>10</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="4" t="s">
-        <v>16</v>
+      <c r="C4" s="2"/>
+      <c r="D4" s="3" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="4" t="s">
-        <v>17</v>
+    <row r="5" spans="2:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-    </row>
-    <row r="7" spans="2:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-    </row>
-    <row r="8" spans="2:4" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-    </row>
-    <row r="9" spans="2:4" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-    </row>
-    <row r="10" spans="2:4" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-    </row>
-    <row r="11" spans="2:4" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-    </row>
-    <row r="12" spans="2:4" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-    </row>
-    <row r="13" spans="2:4" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-    </row>
-    <row r="14" spans="2:4" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-    </row>
-    <row r="15" spans="2:4" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-    </row>
-    <row r="16" spans="2:4" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-    </row>
-    <row r="17" spans="2:4" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-    </row>
-    <row r="18" spans="2:4" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-    </row>
-    <row r="19" spans="2:4" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
+    <row r="6" spans="2:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" spans="2:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.5">
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.5">
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.5">
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.5">
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.5">
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.5">
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.5">
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.5">
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.5">
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.5">
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.5">
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.5">
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -25635,7 +25676,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7516409C-F69E-4E20-9C30-92FF3876415F}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.875" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -25872,15 +25913,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="08a37d9d-9576-4bab-89c6-ad9e0707cb90">
@@ -25891,14 +25923,49 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D42659E-BD4E-470A-BABA-64C3D2E85CDF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D42659E-BD4E-470A-BABA-64C3D2E85CDF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="08a37d9d-9576-4bab-89c6-ad9e0707cb90"/>
+    <ds:schemaRef ds:uri="8e922e2c-d434-4569-88ac-67afeec8ca9b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39A8F35F-7BB6-4037-819F-98AD15F648BF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5E9BDC72-B357-44F6-B254-C90909367FFE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="08a37d9d-9576-4bab-89c6-ad9e0707cb90"/>
+    <ds:schemaRef ds:uri="8e922e2c-d434-4569-88ac-67afeec8ca9b"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5E9BDC72-B357-44F6-B254-C90909367FFE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39A8F35F-7BB6-4037-819F-98AD15F648BF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>